<commit_message>
About page: exhibitions can link to their own website (optional Link column)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDivGFyBfZtVTUyihqwbrz
</commit_message>
<xml_diff>
--- a/sheet-template/fig-tree-studio-website.xlsx
+++ b/sheet-template/fig-tree-studio-website.xlsx
@@ -3043,7 +3043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2"/>
+  <dimension ref="A1:E2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3071,6 +3071,11 @@
       <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Show</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Announcements: a Sheet-driven band under the header (Art Trail first)
New Announcements tab (heading, details, label, button, link, start/end dates,
home-only or all pages). Shown on the main pages; expires by itself.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDivGFyBfZtVTUyihqwbrz
</commit_message>
<xml_diff>
--- a/sheet-template/fig-tree-studio-website.xlsx
+++ b/sheet-template/fig-tree-studio-website.xlsx
@@ -7,11 +7,12 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Workshops" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Studio" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Galleries" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Exhibitions" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Media" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Announcements" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Workshops" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Studio" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Galleries" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Exhibitions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Media" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -434,6 +435,110 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Heading</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Label</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Button text</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Pages</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Show</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Lower Hutt Art Trail, 17–18 October</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Stop 23, Wellington Artspace, 223 The Esplanade, Petone · Free · 10am–4pm both days</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>See Cate's work in person</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Plan your visit</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>https://www.lowerhuttarttrail.co.nz/the_trail/stops.html#stop23</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>18/10/2026</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>All pages</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -684,7 +789,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2929,7 +3034,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3037,7 +3142,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3109,7 +3214,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Homepage gallery list driven by the Galleries tab ("Has Cate's work now")
New galleries need only a Sheet row; ORA and The Vault keep their live piece counts.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GDivGFyBfZtVTUyihqwbrz
</commit_message>
<xml_diff>
--- a/sheet-template/fig-tree-studio-website.xlsx
+++ b/sheet-template/fig-tree-studio-website.xlsx
@@ -511,7 +511,6 @@
           <t>https://www.lowerhuttarttrail.co.nz/the_trail/stops.html#stop23</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>18/10/2026</t>
@@ -3040,7 +3039,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3070,6 +3069,11 @@
           <t>Show</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Has Cate's work now</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -3092,6 +3096,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -3114,6 +3123,11 @@
           <t>yes</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -3129,6 +3143,11 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>yes</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>

</xml_diff>